<commit_message>
docs: use light orange sheet fill and span testing bars
The sheet background is the theme orange at 80% lightness, and Testeo and Documentación run from the first day of each task to the last.

Co-authored-by: Antonio2403 <Antonio2403@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Spartum_Gantt.xlsx
+++ b/docs/Spartum_Gantt.xlsx
@@ -81,7 +81,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999816888943144"/>
+        <fgColor theme="9" tint="0.7999816888943144"/>
       </patternFill>
     </fill>
     <fill>
@@ -463,7 +463,7 @@
         <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
         <a:srgbClr val="4BACC6"/>
@@ -1354,8 +1354,8 @@
           <t>1.4 Testeo</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
       <c r="D12" s="29" t="n"/>
       <c r="E12" s="23" t="n"/>
       <c r="F12" s="23" t="n"/>
@@ -1394,8 +1394,8 @@
           <t>1.5 Documentación</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="23" t="n"/>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="22" t="n"/>
       <c r="D13" s="22" t="n"/>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="23" t="n"/>
@@ -1597,10 +1597,10 @@
       <c r="B18" s="23" t="n"/>
       <c r="C18" s="23" t="n"/>
       <c r="D18" s="23" t="n"/>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="23" t="n"/>
-      <c r="G18" s="23" t="n"/>
-      <c r="H18" s="23" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
+      <c r="G18" s="22" t="n"/>
+      <c r="H18" s="22" t="n"/>
       <c r="I18" s="22" t="n"/>
       <c r="J18" s="23" t="n"/>
       <c r="K18" s="23" t="n"/>
@@ -1637,10 +1637,10 @@
       <c r="B19" s="23" t="n"/>
       <c r="C19" s="23" t="n"/>
       <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="23" t="n"/>
-      <c r="H19" s="23" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="26" t="n"/>
+      <c r="H19" s="26" t="n"/>
       <c r="I19" s="26" t="n"/>
       <c r="J19" s="23" t="n"/>
       <c r="K19" s="23" t="n"/>
@@ -1842,8 +1842,8 @@
       <c r="G24" s="23" t="n"/>
       <c r="H24" s="23" t="n"/>
       <c r="I24" s="23" t="n"/>
-      <c r="J24" s="23" t="n"/>
-      <c r="K24" s="23" t="n"/>
+      <c r="J24" s="26" t="n"/>
+      <c r="K24" s="26" t="n"/>
       <c r="L24" s="26" t="n"/>
       <c r="M24" s="23" t="n"/>
       <c r="N24" s="23" t="n"/>
@@ -1882,8 +1882,8 @@
       <c r="G25" s="23" t="n"/>
       <c r="H25" s="23" t="n"/>
       <c r="I25" s="23" t="n"/>
-      <c r="J25" s="23" t="n"/>
-      <c r="K25" s="23" t="n"/>
+      <c r="J25" s="27" t="n"/>
+      <c r="K25" s="27" t="n"/>
       <c r="L25" s="27" t="n"/>
       <c r="M25" s="23" t="n"/>
       <c r="N25" s="23" t="n"/>
@@ -2085,9 +2085,9 @@
       <c r="J30" s="23" t="n"/>
       <c r="K30" s="23" t="n"/>
       <c r="L30" s="23" t="n"/>
-      <c r="M30" s="23" t="n"/>
-      <c r="N30" s="23" t="n"/>
-      <c r="O30" s="23" t="n"/>
+      <c r="M30" s="27" t="n"/>
+      <c r="N30" s="27" t="n"/>
+      <c r="O30" s="27" t="n"/>
       <c r="P30" s="27" t="n"/>
       <c r="Q30" s="23" t="n"/>
       <c r="R30" s="23" t="n"/>
@@ -2125,9 +2125,9 @@
       <c r="J31" s="23" t="n"/>
       <c r="K31" s="23" t="n"/>
       <c r="L31" s="23" t="n"/>
-      <c r="M31" s="23" t="n"/>
-      <c r="N31" s="23" t="n"/>
-      <c r="O31" s="23" t="n"/>
+      <c r="M31" s="28" t="n"/>
+      <c r="N31" s="28" t="n"/>
+      <c r="O31" s="28" t="n"/>
       <c r="P31" s="28" t="n"/>
       <c r="Q31" s="23" t="n"/>
       <c r="R31" s="23" t="n"/>
@@ -2329,8 +2329,8 @@
       <c r="N36" s="23" t="n"/>
       <c r="O36" s="23" t="n"/>
       <c r="P36" s="23" t="n"/>
-      <c r="Q36" s="23" t="n"/>
-      <c r="R36" s="23" t="n"/>
+      <c r="Q36" s="28" t="n"/>
+      <c r="R36" s="28" t="n"/>
       <c r="S36" s="28" t="n"/>
       <c r="T36" s="23" t="n"/>
       <c r="U36" s="23" t="n"/>
@@ -2342,9 +2342,9 @@
       <c r="AA36" s="23" t="n"/>
       <c r="AB36" s="23" t="n"/>
       <c r="AC36" s="23" t="n"/>
-      <c r="AD36" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD36" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2369,8 +2369,8 @@
       <c r="N37" s="23" t="n"/>
       <c r="O37" s="23" t="n"/>
       <c r="P37" s="23" t="n"/>
-      <c r="Q37" s="23" t="n"/>
-      <c r="R37" s="23" t="n"/>
+      <c r="Q37" s="29" t="n"/>
+      <c r="R37" s="29" t="n"/>
       <c r="S37" s="29" t="n"/>
       <c r="T37" s="23" t="n"/>
       <c r="U37" s="23" t="n"/>
@@ -2382,9 +2382,9 @@
       <c r="AA37" s="23" t="n"/>
       <c r="AB37" s="23" t="n"/>
       <c r="AC37" s="23" t="n"/>
-      <c r="AD37" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD37" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2572,10 +2572,10 @@
       <c r="Q42" s="23" t="n"/>
       <c r="R42" s="23" t="n"/>
       <c r="S42" s="23" t="n"/>
-      <c r="T42" s="23" t="n"/>
-      <c r="U42" s="23" t="n"/>
-      <c r="V42" s="23" t="n"/>
-      <c r="W42" s="23" t="n"/>
+      <c r="T42" s="29" t="n"/>
+      <c r="U42" s="29" t="n"/>
+      <c r="V42" s="29" t="n"/>
+      <c r="W42" s="29" t="n"/>
       <c r="X42" s="29" t="n"/>
       <c r="Y42" s="23" t="n"/>
       <c r="Z42" s="23" t="n"/>
@@ -2612,10 +2612,10 @@
       <c r="Q43" s="23" t="n"/>
       <c r="R43" s="23" t="n"/>
       <c r="S43" s="23" t="n"/>
-      <c r="T43" s="23" t="n"/>
-      <c r="U43" s="23" t="n"/>
-      <c r="V43" s="23" t="n"/>
-      <c r="W43" s="23" t="n"/>
+      <c r="T43" s="22" t="n"/>
+      <c r="U43" s="22" t="n"/>
+      <c r="V43" s="22" t="n"/>
+      <c r="W43" s="22" t="n"/>
       <c r="X43" s="22" t="n"/>
       <c r="Y43" s="23" t="n"/>
       <c r="Z43" s="23" t="n"/>
@@ -2817,7 +2817,7 @@
       <c r="V48" s="23" t="n"/>
       <c r="W48" s="23" t="n"/>
       <c r="X48" s="23" t="n"/>
-      <c r="Y48" s="23" t="n"/>
+      <c r="Y48" s="22" t="n"/>
       <c r="Z48" s="22" t="n"/>
       <c r="AA48" s="23" t="n"/>
       <c r="AB48" s="23" t="n"/>
@@ -2857,7 +2857,7 @@
       <c r="V49" s="23" t="n"/>
       <c r="W49" s="23" t="n"/>
       <c r="X49" s="23" t="n"/>
-      <c r="Y49" s="23" t="n"/>
+      <c r="Y49" s="26" t="n"/>
       <c r="Z49" s="26" t="n"/>
       <c r="AA49" s="23" t="n"/>
       <c r="AB49" s="23" t="n"/>
@@ -3059,9 +3059,9 @@
       <c r="X54" s="23" t="n"/>
       <c r="Y54" s="23" t="n"/>
       <c r="Z54" s="23" t="n"/>
-      <c r="AA54" s="23" t="n"/>
-      <c r="AB54" s="23" t="n"/>
-      <c r="AC54" s="23" t="n"/>
+      <c r="AA54" s="26" t="n"/>
+      <c r="AB54" s="26" t="n"/>
+      <c r="AC54" s="26" t="n"/>
       <c r="AD54" s="31" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -3099,9 +3099,9 @@
       <c r="X55" s="23" t="n"/>
       <c r="Y55" s="23" t="n"/>
       <c r="Z55" s="23" t="n"/>
-      <c r="AA55" s="23" t="n"/>
-      <c r="AB55" s="23" t="n"/>
-      <c r="AC55" s="23" t="n"/>
+      <c r="AA55" s="27" t="n"/>
+      <c r="AB55" s="27" t="n"/>
+      <c r="AC55" s="27" t="n"/>
       <c r="AD55" s="31" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -6559,9 +6559,9 @@
       <c r="AA36" s="23" t="n"/>
       <c r="AB36" s="23" t="n"/>
       <c r="AC36" s="23" t="n"/>
-      <c r="AD36" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD36" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6599,9 +6599,9 @@
       <c r="AA37" s="23" t="n"/>
       <c r="AB37" s="23" t="n"/>
       <c r="AC37" s="23" t="n"/>
-      <c r="AD37" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD37" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
           <t>8.4 Testeo</t>
         </is>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="26" t="n"/>
       <c r="C54" s="26" t="n"/>
       <c r="D54" s="23" t="n"/>
       <c r="E54" s="23" t="n"/>
@@ -7291,7 +7291,7 @@
           <t>8.5 Documentación</t>
         </is>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="27" t="n"/>
       <c r="C55" s="27" t="n"/>
       <c r="D55" s="23" t="n"/>
       <c r="E55" s="23" t="n"/>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="B60" s="23" t="n"/>
       <c r="C60" s="23" t="n"/>
-      <c r="D60" s="23" t="n"/>
+      <c r="D60" s="27" t="n"/>
       <c r="E60" s="27" t="n"/>
       <c r="F60" s="23" t="n"/>
       <c r="G60" s="23" t="n"/>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B61" s="23" t="n"/>
       <c r="C61" s="23" t="n"/>
-      <c r="D61" s="23" t="n"/>
+      <c r="D61" s="28" t="n"/>
       <c r="E61" s="28" t="n"/>
       <c r="F61" s="23" t="n"/>
       <c r="G61" s="23" t="n"/>
@@ -7735,9 +7735,9 @@
       <c r="C66" s="23" t="n"/>
       <c r="D66" s="23" t="n"/>
       <c r="E66" s="23" t="n"/>
-      <c r="F66" s="23" t="n"/>
-      <c r="G66" s="23" t="n"/>
-      <c r="H66" s="23" t="n"/>
+      <c r="F66" s="28" t="n"/>
+      <c r="G66" s="28" t="n"/>
+      <c r="H66" s="28" t="n"/>
       <c r="I66" s="28" t="n"/>
       <c r="J66" s="23" t="n"/>
       <c r="K66" s="23" t="n"/>
@@ -7775,9 +7775,9 @@
       <c r="C67" s="23" t="n"/>
       <c r="D67" s="23" t="n"/>
       <c r="E67" s="23" t="n"/>
-      <c r="F67" s="23" t="n"/>
-      <c r="G67" s="23" t="n"/>
-      <c r="H67" s="23" t="n"/>
+      <c r="F67" s="29" t="n"/>
+      <c r="G67" s="29" t="n"/>
+      <c r="H67" s="29" t="n"/>
       <c r="I67" s="29" t="n"/>
       <c r="J67" s="23" t="n"/>
       <c r="K67" s="23" t="n"/>
@@ -7979,8 +7979,8 @@
       <c r="G72" s="23" t="n"/>
       <c r="H72" s="23" t="n"/>
       <c r="I72" s="23" t="n"/>
-      <c r="J72" s="23" t="n"/>
-      <c r="K72" s="23" t="n"/>
+      <c r="J72" s="29" t="n"/>
+      <c r="K72" s="29" t="n"/>
       <c r="L72" s="29" t="n"/>
       <c r="M72" s="23" t="n"/>
       <c r="N72" s="23" t="n"/>
@@ -8019,8 +8019,8 @@
       <c r="G73" s="23" t="n"/>
       <c r="H73" s="23" t="n"/>
       <c r="I73" s="23" t="n"/>
-      <c r="J73" s="23" t="n"/>
-      <c r="K73" s="23" t="n"/>
+      <c r="J73" s="22" t="n"/>
+      <c r="K73" s="22" t="n"/>
       <c r="L73" s="22" t="n"/>
       <c r="M73" s="23" t="n"/>
       <c r="N73" s="23" t="n"/>
@@ -8222,9 +8222,9 @@
       <c r="J78" s="23" t="n"/>
       <c r="K78" s="23" t="n"/>
       <c r="L78" s="23" t="n"/>
-      <c r="M78" s="23" t="n"/>
-      <c r="N78" s="23" t="n"/>
-      <c r="O78" s="23" t="n"/>
+      <c r="M78" s="22" t="n"/>
+      <c r="N78" s="22" t="n"/>
+      <c r="O78" s="22" t="n"/>
       <c r="P78" s="22" t="n"/>
       <c r="Q78" s="23" t="n"/>
       <c r="R78" s="23" t="n"/>
@@ -8262,9 +8262,9 @@
       <c r="J79" s="23" t="n"/>
       <c r="K79" s="23" t="n"/>
       <c r="L79" s="23" t="n"/>
-      <c r="M79" s="23" t="n"/>
-      <c r="N79" s="23" t="n"/>
-      <c r="O79" s="23" t="n"/>
+      <c r="M79" s="26" t="n"/>
+      <c r="N79" s="26" t="n"/>
+      <c r="O79" s="26" t="n"/>
       <c r="P79" s="26" t="n"/>
       <c r="Q79" s="23" t="n"/>
       <c r="R79" s="23" t="n"/>
@@ -8466,8 +8466,8 @@
       <c r="N84" s="23" t="n"/>
       <c r="O84" s="23" t="n"/>
       <c r="P84" s="23" t="n"/>
-      <c r="Q84" s="23" t="n"/>
-      <c r="R84" s="23" t="n"/>
+      <c r="Q84" s="26" t="n"/>
+      <c r="R84" s="26" t="n"/>
       <c r="S84" s="26" t="n"/>
       <c r="T84" s="23" t="n"/>
       <c r="U84" s="23" t="n"/>
@@ -8506,8 +8506,8 @@
       <c r="N85" s="23" t="n"/>
       <c r="O85" s="23" t="n"/>
       <c r="P85" s="23" t="n"/>
-      <c r="Q85" s="23" t="n"/>
-      <c r="R85" s="23" t="n"/>
+      <c r="Q85" s="27" t="n"/>
+      <c r="R85" s="27" t="n"/>
       <c r="S85" s="27" t="n"/>
       <c r="T85" s="23" t="n"/>
       <c r="U85" s="23" t="n"/>
@@ -8709,10 +8709,10 @@
       <c r="Q90" s="23" t="n"/>
       <c r="R90" s="23" t="n"/>
       <c r="S90" s="23" t="n"/>
-      <c r="T90" s="23" t="n"/>
-      <c r="U90" s="23" t="n"/>
-      <c r="V90" s="23" t="n"/>
-      <c r="W90" s="23" t="n"/>
+      <c r="T90" s="27" t="n"/>
+      <c r="U90" s="27" t="n"/>
+      <c r="V90" s="27" t="n"/>
+      <c r="W90" s="27" t="n"/>
       <c r="X90" s="27" t="n"/>
       <c r="Y90" s="23" t="n"/>
       <c r="Z90" s="23" t="n"/>
@@ -8749,10 +8749,10 @@
       <c r="Q91" s="23" t="n"/>
       <c r="R91" s="23" t="n"/>
       <c r="S91" s="23" t="n"/>
-      <c r="T91" s="23" t="n"/>
-      <c r="U91" s="23" t="n"/>
-      <c r="V91" s="23" t="n"/>
-      <c r="W91" s="23" t="n"/>
+      <c r="T91" s="28" t="n"/>
+      <c r="U91" s="28" t="n"/>
+      <c r="V91" s="28" t="n"/>
+      <c r="W91" s="28" t="n"/>
       <c r="X91" s="28" t="n"/>
       <c r="Y91" s="23" t="n"/>
       <c r="Z91" s="23" t="n"/>
@@ -8954,8 +8954,8 @@
       <c r="V96" s="23" t="n"/>
       <c r="W96" s="23" t="n"/>
       <c r="X96" s="23" t="n"/>
-      <c r="Y96" s="23" t="n"/>
-      <c r="Z96" s="23" t="n"/>
+      <c r="Y96" s="28" t="n"/>
+      <c r="Z96" s="28" t="n"/>
       <c r="AA96" s="28" t="n"/>
       <c r="AB96" s="28" t="n"/>
       <c r="AC96" s="28" t="n"/>
@@ -8994,8 +8994,8 @@
       <c r="V97" s="23" t="n"/>
       <c r="W97" s="23" t="n"/>
       <c r="X97" s="23" t="n"/>
-      <c r="Y97" s="23" t="n"/>
-      <c r="Z97" s="23" t="n"/>
+      <c r="Y97" s="29" t="n"/>
+      <c r="Z97" s="29" t="n"/>
       <c r="AA97" s="29" t="n"/>
       <c r="AB97" s="29" t="n"/>
       <c r="AC97" s="29" t="n"/>
@@ -10481,9 +10481,9 @@
       <c r="T36" s="23" t="n"/>
       <c r="U36" s="23" t="n"/>
       <c r="V36" s="23" t="n"/>
-      <c r="W36" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W36" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10514,9 +10514,9 @@
       <c r="T37" s="23" t="n"/>
       <c r="U37" s="23" t="n"/>
       <c r="V37" s="23" t="n"/>
-      <c r="W37" s="31" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W37" s="30" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -12474,10 +12474,10 @@
         </is>
       </c>
       <c r="B97" s="29" t="n"/>
-      <c r="C97" s="23" t="n"/>
-      <c r="D97" s="23" t="n"/>
-      <c r="E97" s="23" t="n"/>
-      <c r="F97" s="23" t="n"/>
+      <c r="C97" s="29" t="n"/>
+      <c r="D97" s="29" t="n"/>
+      <c r="E97" s="29" t="n"/>
+      <c r="F97" s="29" t="n"/>
       <c r="G97" s="23" t="n"/>
       <c r="H97" s="23" t="n"/>
       <c r="I97" s="23" t="n"/>

</xml_diff>

<commit_message>
docs: place the 2-6 November review on the existing Gantt tasks
The review notes stay on the modules that already own them, on the day
each one is worked, without adding new tasks.

Co-authored-by: Antonio2403 <Antonio2403@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Spartum_Gantt.xlsx
+++ b/docs/Spartum_Gantt.xlsx
@@ -11,11 +11,7 @@
     <sheet name="Planificación Mes 2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Planificación Mes 3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Planificación Mes 1'!$A$1:$AD$101</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planificación Mes 2'!$A$1:$AD$101</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Planificación Mes 3'!$A$1:$W$101</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -33,6 +29,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FF0000"/>
       <sz val="22"/>
@@ -42,11 +43,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -95,9 +91,6 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid"/>
-    </fill>
-    <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EC5E61"/>
       </patternFill>
@@ -111,6 +104,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="00008000"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -201,83 +197,6 @@
       </bottom>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00F4883C"/>
       </left>
@@ -347,29 +266,106 @@
         <color rgb="00FAE29C"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -379,11 +375,11 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -395,44 +391,44 @@
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -802,7 +798,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AD101"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="3.7" customWidth="1" min="2" max="2"/>
@@ -1972,9 +1968,9 @@
       <c r="AA26" s="22" t="n"/>
       <c r="AB26" s="22" t="n"/>
       <c r="AC26" s="22" t="n"/>
-      <c r="AD26" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD26" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2057,7 @@
     <row r="29" outlineLevel="1" ht="14" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>4.3 Baja y reactivación</t>
+          <t>4.3 Baja: al redirigir se pierde la sesión</t>
         </is>
       </c>
       <c r="B29" s="22" t="n"/>
@@ -2092,9 +2088,9 @@
       <c r="AA29" s="22" t="n"/>
       <c r="AB29" s="22" t="n"/>
       <c r="AC29" s="22" t="n"/>
-      <c r="AD29" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD29" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2132,9 +2128,9 @@
       <c r="AA30" s="22" t="n"/>
       <c r="AB30" s="22" t="n"/>
       <c r="AC30" s="22" t="n"/>
-      <c r="AD30" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD30" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2172,9 +2168,9 @@
       <c r="AA31" s="22" t="n"/>
       <c r="AB31" s="22" t="n"/>
       <c r="AC31" s="22" t="n"/>
-      <c r="AD31" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD31" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2217,7 @@
     <row r="33" outlineLevel="1" ht="14" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>5.1 Listado de actividades</t>
+          <t>5.1 Listado descuadrado</t>
         </is>
       </c>
       <c r="B33" s="22" t="n"/>
@@ -2252,16 +2248,16 @@
       <c r="AA33" s="22" t="n"/>
       <c r="AB33" s="22" t="n"/>
       <c r="AC33" s="22" t="n"/>
-      <c r="AD33" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD33" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
     <row r="34" outlineLevel="1" ht="14" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>5.2 Horario y avisos → inscritos</t>
+          <t>5.2 Horario con uniformidad</t>
         </is>
       </c>
       <c r="B34" s="22" t="n"/>
@@ -2292,9 +2288,9 @@
       <c r="AA34" s="22" t="n"/>
       <c r="AB34" s="22" t="n"/>
       <c r="AC34" s="22" t="n"/>
-      <c r="AD34" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD34" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -2332,9 +2328,9 @@
       <c r="AA35" s="22" t="n"/>
       <c r="AB35" s="22" t="n"/>
       <c r="AC35" s="22" t="n"/>
-      <c r="AD35" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD35" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2692,9 +2688,9 @@
       <c r="AA44" s="22" t="n"/>
       <c r="AB44" s="22" t="n"/>
       <c r="AC44" s="22" t="n"/>
-      <c r="AD44" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD44" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2732,9 +2728,9 @@
       <c r="AA45" s="22" t="n"/>
       <c r="AB45" s="22" t="n"/>
       <c r="AC45" s="22" t="n"/>
-      <c r="AD45" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD45" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2772,9 +2768,9 @@
       <c r="AA46" s="22" t="n"/>
       <c r="AB46" s="22" t="n"/>
       <c r="AC46" s="22" t="n"/>
-      <c r="AD46" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD46" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2812,9 +2808,9 @@
       <c r="AA47" s="22" t="n"/>
       <c r="AB47" s="22" t="n"/>
       <c r="AC47" s="22" t="n"/>
-      <c r="AD47" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD47" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2852,9 +2848,9 @@
       <c r="AA48" s="22" t="n"/>
       <c r="AB48" s="22" t="n"/>
       <c r="AC48" s="22" t="n"/>
-      <c r="AD48" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD48" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2892,9 +2888,9 @@
       <c r="AA49" s="22" t="n"/>
       <c r="AB49" s="22" t="n"/>
       <c r="AC49" s="22" t="n"/>
-      <c r="AD49" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD49" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2977,7 @@
     <row r="52" outlineLevel="1" ht="14" customHeight="1">
       <c r="A52" s="24" t="inlineStr">
         <is>
-          <t>8.2 Confirmación del pago</t>
+          <t>8.2 Guardar el método de pago</t>
         </is>
       </c>
       <c r="B52" s="22" t="n"/>
@@ -3181,7 +3177,7 @@
     <row r="57" outlineLevel="1" ht="14" customHeight="1">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>9.1 Inicio del panel</t>
+          <t>9.1 Vista de admin descuadrada</t>
         </is>
       </c>
       <c r="B57" s="22" t="n"/>
@@ -3501,7 +3497,7 @@
     <row r="65" outlineLevel="1" ht="14" customHeight="1">
       <c r="A65" s="24" t="inlineStr">
         <is>
-          <t>10.3 Edición de datos</t>
+          <t>10.3 Impersonalidad: usuario1</t>
         </is>
       </c>
       <c r="B65" s="22" t="n"/>
@@ -3621,7 +3617,7 @@
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="20" t="inlineStr">
         <is>
-          <t>11. Monitores y solicitudes</t>
+          <t>11. Monitores y reportes</t>
         </is>
       </c>
       <c r="B68" s="22" t="n"/>
@@ -3661,7 +3657,7 @@
     <row r="69" outlineLevel="1" ht="14" customHeight="1">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t>11.1 Alta de monitores</t>
+          <t>11.1 Impersonalidad: monitor1</t>
         </is>
       </c>
       <c r="B69" s="22" t="n"/>
@@ -3701,7 +3697,7 @@
     <row r="70" outlineLevel="1" ht="14" customHeight="1">
       <c r="A70" s="24" t="inlineStr">
         <is>
-          <t>11.2 Solicitudes de clase</t>
+          <t>11.2 De solicitudes a reportes</t>
         </is>
       </c>
       <c r="B70" s="22" t="n"/>
@@ -3901,7 +3897,7 @@
     <row r="75" outlineLevel="1" ht="14" customHeight="1">
       <c r="A75" s="24" t="inlineStr">
         <is>
-          <t>12.1 Ficha de salas</t>
+          <t>12.1 Colores de salas y actividades</t>
         </is>
       </c>
       <c r="B75" s="22" t="n"/>
@@ -4652,9 +4648,9 @@
       <c r="AA93" s="22" t="n"/>
       <c r="AB93" s="22" t="n"/>
       <c r="AC93" s="22" t="n"/>
-      <c r="AD93" s="29" t="inlineStr">
-        <is>
-          <t>en curso</t>
+      <c r="AD93" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -4692,9 +4688,9 @@
       <c r="AA94" s="25" t="n"/>
       <c r="AB94" s="22" t="n"/>
       <c r="AC94" s="22" t="n"/>
-      <c r="AD94" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD94" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -4952,12 +4948,12 @@
     <mergeCell ref="I5:O5"/>
     <mergeCell ref="P5:V5"/>
     <mergeCell ref="W4:AC4"/>
+    <mergeCell ref="AD4:AD7"/>
+    <mergeCell ref="B4:H4"/>
     <mergeCell ref="W5:AC5"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="AD4:AD7"/>
     <mergeCell ref="P4:V4"/>
+    <mergeCell ref="A2:AD2"/>
     <mergeCell ref="I4:O4"/>
-    <mergeCell ref="A2:AD2"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
@@ -4975,7 +4971,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AD101"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="3.7" customWidth="1" min="2" max="2"/>
@@ -6117,7 +6113,7 @@
           <t>4. Perfil, contraseña y baja</t>
         </is>
       </c>
-      <c r="B26" s="22" t="n"/>
+      <c r="B26" s="27" t="n"/>
       <c r="C26" s="22" t="n"/>
       <c r="D26" s="22" t="n"/>
       <c r="E26" s="22" t="n"/>
@@ -6145,9 +6141,9 @@
       <c r="AA26" s="22" t="n"/>
       <c r="AB26" s="22" t="n"/>
       <c r="AC26" s="22" t="n"/>
-      <c r="AD26" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD26" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6234,10 +6230,10 @@
     <row r="29" outlineLevel="1" ht="14" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>4.3 Baja y reactivación</t>
-        </is>
-      </c>
-      <c r="B29" s="22" t="n"/>
+          <t>4.3 Baja: al redirigir se pierde la sesión</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n"/>
       <c r="C29" s="22" t="n"/>
       <c r="D29" s="22" t="n"/>
       <c r="E29" s="22" t="n"/>
@@ -6265,9 +6261,9 @@
       <c r="AA29" s="22" t="n"/>
       <c r="AB29" s="22" t="n"/>
       <c r="AC29" s="22" t="n"/>
-      <c r="AD29" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD29" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6273,7 @@
           <t>4.4 Testeo</t>
         </is>
       </c>
-      <c r="B30" s="22" t="n"/>
+      <c r="B30" s="26" t="n"/>
       <c r="C30" s="22" t="n"/>
       <c r="D30" s="22" t="n"/>
       <c r="E30" s="22" t="n"/>
@@ -6305,9 +6301,9 @@
       <c r="AA30" s="22" t="n"/>
       <c r="AB30" s="22" t="n"/>
       <c r="AC30" s="22" t="n"/>
-      <c r="AD30" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD30" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6317,7 +6313,7 @@
           <t>4.5 Documentación</t>
         </is>
       </c>
-      <c r="B31" s="22" t="n"/>
+      <c r="B31" s="27" t="n"/>
       <c r="C31" s="22" t="n"/>
       <c r="D31" s="22" t="n"/>
       <c r="E31" s="22" t="n"/>
@@ -6345,9 +6341,9 @@
       <c r="AA31" s="22" t="n"/>
       <c r="AB31" s="22" t="n"/>
       <c r="AC31" s="22" t="n"/>
-      <c r="AD31" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD31" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6360,8 +6356,8 @@
       <c r="B32" s="22" t="n"/>
       <c r="C32" s="22" t="n"/>
       <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
-      <c r="F32" s="22" t="n"/>
+      <c r="E32" s="28" t="n"/>
+      <c r="F32" s="28" t="n"/>
       <c r="G32" s="22" t="n"/>
       <c r="H32" s="22" t="n"/>
       <c r="I32" s="22" t="n"/>
@@ -6394,13 +6390,13 @@
     <row r="33" outlineLevel="1" ht="14" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>5.1 Listado de actividades</t>
+          <t>5.1 Listado descuadrado</t>
         </is>
       </c>
       <c r="B33" s="22" t="n"/>
       <c r="C33" s="22" t="n"/>
       <c r="D33" s="22" t="n"/>
-      <c r="E33" s="22" t="n"/>
+      <c r="E33" s="21" t="n"/>
       <c r="F33" s="22" t="n"/>
       <c r="G33" s="22" t="n"/>
       <c r="H33" s="22" t="n"/>
@@ -6425,23 +6421,23 @@
       <c r="AA33" s="22" t="n"/>
       <c r="AB33" s="22" t="n"/>
       <c r="AC33" s="22" t="n"/>
-      <c r="AD33" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD33" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
     <row r="34" outlineLevel="1" ht="14" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>5.2 Horario y avisos → inscritos</t>
+          <t>5.2 Horario con uniformidad</t>
         </is>
       </c>
       <c r="B34" s="22" t="n"/>
       <c r="C34" s="22" t="n"/>
       <c r="D34" s="22" t="n"/>
       <c r="E34" s="22" t="n"/>
-      <c r="F34" s="22" t="n"/>
+      <c r="F34" s="25" t="n"/>
       <c r="G34" s="22" t="n"/>
       <c r="H34" s="22" t="n"/>
       <c r="I34" s="22" t="n"/>
@@ -6465,9 +6461,9 @@
       <c r="AA34" s="22" t="n"/>
       <c r="AB34" s="22" t="n"/>
       <c r="AC34" s="22" t="n"/>
-      <c r="AD34" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="AD34" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -6505,9 +6501,9 @@
       <c r="AA35" s="22" t="n"/>
       <c r="AB35" s="22" t="n"/>
       <c r="AC35" s="22" t="n"/>
-      <c r="AD35" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD35" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -6520,8 +6516,8 @@
       <c r="B36" s="22" t="n"/>
       <c r="C36" s="22" t="n"/>
       <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="22" t="n"/>
+      <c r="E36" s="27" t="n"/>
+      <c r="F36" s="27" t="n"/>
       <c r="G36" s="22" t="n"/>
       <c r="H36" s="22" t="n"/>
       <c r="I36" s="22" t="n"/>
@@ -6560,8 +6556,8 @@
       <c r="B37" s="22" t="n"/>
       <c r="C37" s="22" t="n"/>
       <c r="D37" s="22" t="n"/>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="22" t="n"/>
+      <c r="E37" s="28" t="n"/>
+      <c r="F37" s="28" t="n"/>
       <c r="G37" s="22" t="n"/>
       <c r="H37" s="22" t="n"/>
       <c r="I37" s="22" t="n"/>
@@ -6597,18 +6593,18 @@
           <t>6. Inscripciones y reservas</t>
         </is>
       </c>
-      <c r="B38" s="21" t="n"/>
-      <c r="C38" s="21" t="n"/>
-      <c r="D38" s="21" t="n"/>
-      <c r="E38" s="21" t="n"/>
-      <c r="F38" s="21" t="n"/>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="22" t="n"/>
       <c r="G38" s="22" t="n"/>
       <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
-      <c r="J38" s="22" t="n"/>
-      <c r="K38" s="22" t="n"/>
-      <c r="L38" s="22" t="n"/>
-      <c r="M38" s="22" t="n"/>
+      <c r="I38" s="21" t="n"/>
+      <c r="J38" s="21" t="n"/>
+      <c r="K38" s="21" t="n"/>
+      <c r="L38" s="21" t="n"/>
+      <c r="M38" s="21" t="n"/>
       <c r="N38" s="22" t="n"/>
       <c r="O38" s="22" t="n"/>
       <c r="P38" s="22" t="n"/>
@@ -6637,14 +6633,14 @@
           <t>6.1 Formulario de inscripción</t>
         </is>
       </c>
-      <c r="B39" s="25" t="n"/>
+      <c r="B39" s="22" t="n"/>
       <c r="C39" s="22" t="n"/>
       <c r="D39" s="22" t="n"/>
       <c r="E39" s="22" t="n"/>
       <c r="F39" s="22" t="n"/>
       <c r="G39" s="22" t="n"/>
       <c r="H39" s="22" t="n"/>
-      <c r="I39" s="22" t="n"/>
+      <c r="I39" s="25" t="n"/>
       <c r="J39" s="22" t="n"/>
       <c r="K39" s="22" t="n"/>
       <c r="L39" s="22" t="n"/>
@@ -6680,14 +6676,14 @@
       <c r="B40" s="22" t="n"/>
       <c r="C40" s="22" t="n"/>
       <c r="D40" s="22" t="n"/>
-      <c r="E40" s="26" t="n"/>
+      <c r="E40" s="22" t="n"/>
       <c r="F40" s="22" t="n"/>
       <c r="G40" s="22" t="n"/>
       <c r="H40" s="22" t="n"/>
       <c r="I40" s="22" t="n"/>
       <c r="J40" s="22" t="n"/>
       <c r="K40" s="22" t="n"/>
-      <c r="L40" s="22" t="n"/>
+      <c r="L40" s="26" t="n"/>
       <c r="M40" s="22" t="n"/>
       <c r="N40" s="22" t="n"/>
       <c r="O40" s="22" t="n"/>
@@ -6720,14 +6716,14 @@
       <c r="B41" s="22" t="n"/>
       <c r="C41" s="22" t="n"/>
       <c r="D41" s="22" t="n"/>
-      <c r="E41" s="27" t="n"/>
+      <c r="E41" s="22" t="n"/>
       <c r="F41" s="22" t="n"/>
       <c r="G41" s="22" t="n"/>
       <c r="H41" s="22" t="n"/>
       <c r="I41" s="22" t="n"/>
       <c r="J41" s="22" t="n"/>
       <c r="K41" s="22" t="n"/>
-      <c r="L41" s="22" t="n"/>
+      <c r="L41" s="27" t="n"/>
       <c r="M41" s="22" t="n"/>
       <c r="N41" s="22" t="n"/>
       <c r="O41" s="22" t="n"/>
@@ -6757,18 +6753,18 @@
           <t>6.4 Testeo</t>
         </is>
       </c>
-      <c r="B42" s="28" t="n"/>
-      <c r="C42" s="28" t="n"/>
-      <c r="D42" s="28" t="n"/>
-      <c r="E42" s="28" t="n"/>
-      <c r="F42" s="28" t="n"/>
+      <c r="B42" s="22" t="n"/>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="22" t="n"/>
+      <c r="E42" s="22" t="n"/>
+      <c r="F42" s="22" t="n"/>
       <c r="G42" s="22" t="n"/>
       <c r="H42" s="22" t="n"/>
-      <c r="I42" s="22" t="n"/>
-      <c r="J42" s="22" t="n"/>
-      <c r="K42" s="22" t="n"/>
-      <c r="L42" s="22" t="n"/>
-      <c r="M42" s="22" t="n"/>
+      <c r="I42" s="28" t="n"/>
+      <c r="J42" s="28" t="n"/>
+      <c r="K42" s="28" t="n"/>
+      <c r="L42" s="28" t="n"/>
+      <c r="M42" s="28" t="n"/>
       <c r="N42" s="22" t="n"/>
       <c r="O42" s="22" t="n"/>
       <c r="P42" s="22" t="n"/>
@@ -6797,18 +6793,18 @@
           <t>6.5 Documentación</t>
         </is>
       </c>
-      <c r="B43" s="21" t="n"/>
-      <c r="C43" s="21" t="n"/>
-      <c r="D43" s="21" t="n"/>
-      <c r="E43" s="21" t="n"/>
-      <c r="F43" s="21" t="n"/>
+      <c r="B43" s="22" t="n"/>
+      <c r="C43" s="22" t="n"/>
+      <c r="D43" s="22" t="n"/>
+      <c r="E43" s="22" t="n"/>
+      <c r="F43" s="22" t="n"/>
       <c r="G43" s="22" t="n"/>
       <c r="H43" s="22" t="n"/>
-      <c r="I43" s="22" t="n"/>
-      <c r="J43" s="22" t="n"/>
-      <c r="K43" s="22" t="n"/>
-      <c r="L43" s="22" t="n"/>
-      <c r="M43" s="22" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
+      <c r="L43" s="21" t="n"/>
+      <c r="M43" s="21" t="n"/>
       <c r="N43" s="22" t="n"/>
       <c r="O43" s="22" t="n"/>
       <c r="P43" s="22" t="n"/>
@@ -6865,9 +6861,9 @@
       <c r="AA44" s="22" t="n"/>
       <c r="AB44" s="22" t="n"/>
       <c r="AC44" s="22" t="n"/>
-      <c r="AD44" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD44" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -6905,9 +6901,9 @@
       <c r="AA45" s="22" t="n"/>
       <c r="AB45" s="22" t="n"/>
       <c r="AC45" s="22" t="n"/>
-      <c r="AD45" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD45" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -6945,9 +6941,9 @@
       <c r="AA46" s="22" t="n"/>
       <c r="AB46" s="22" t="n"/>
       <c r="AC46" s="22" t="n"/>
-      <c r="AD46" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD46" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -6985,9 +6981,9 @@
       <c r="AA47" s="22" t="n"/>
       <c r="AB47" s="22" t="n"/>
       <c r="AC47" s="22" t="n"/>
-      <c r="AD47" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD47" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -7025,9 +7021,9 @@
       <c r="AA48" s="22" t="n"/>
       <c r="AB48" s="22" t="n"/>
       <c r="AC48" s="22" t="n"/>
-      <c r="AD48" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD48" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -7065,9 +7061,9 @@
       <c r="AA49" s="22" t="n"/>
       <c r="AB49" s="22" t="n"/>
       <c r="AC49" s="22" t="n"/>
-      <c r="AD49" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD49" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -7078,24 +7074,24 @@
         </is>
       </c>
       <c r="B50" s="22" t="n"/>
-      <c r="C50" s="22" t="n"/>
+      <c r="C50" s="26" t="n"/>
       <c r="D50" s="22" t="n"/>
       <c r="E50" s="22" t="n"/>
       <c r="F50" s="22" t="n"/>
       <c r="G50" s="22" t="n"/>
       <c r="H50" s="22" t="n"/>
-      <c r="I50" s="26" t="n"/>
-      <c r="J50" s="26" t="n"/>
-      <c r="K50" s="26" t="n"/>
-      <c r="L50" s="26" t="n"/>
-      <c r="M50" s="26" t="n"/>
+      <c r="I50" s="22" t="n"/>
+      <c r="J50" s="22" t="n"/>
+      <c r="K50" s="22" t="n"/>
+      <c r="L50" s="22" t="n"/>
+      <c r="M50" s="22" t="n"/>
       <c r="N50" s="22" t="n"/>
       <c r="O50" s="22" t="n"/>
-      <c r="P50" s="22" t="n"/>
-      <c r="Q50" s="22" t="n"/>
-      <c r="R50" s="22" t="n"/>
-      <c r="S50" s="22" t="n"/>
-      <c r="T50" s="22" t="n"/>
+      <c r="P50" s="26" t="n"/>
+      <c r="Q50" s="26" t="n"/>
+      <c r="R50" s="26" t="n"/>
+      <c r="S50" s="26" t="n"/>
+      <c r="T50" s="26" t="n"/>
       <c r="U50" s="22" t="n"/>
       <c r="V50" s="22" t="n"/>
       <c r="W50" s="22" t="n"/>
@@ -7124,14 +7120,14 @@
       <c r="F51" s="22" t="n"/>
       <c r="G51" s="22" t="n"/>
       <c r="H51" s="22" t="n"/>
-      <c r="I51" s="27" t="n"/>
+      <c r="I51" s="22" t="n"/>
       <c r="J51" s="22" t="n"/>
       <c r="K51" s="22" t="n"/>
       <c r="L51" s="22" t="n"/>
       <c r="M51" s="22" t="n"/>
       <c r="N51" s="22" t="n"/>
       <c r="O51" s="22" t="n"/>
-      <c r="P51" s="22" t="n"/>
+      <c r="P51" s="27" t="n"/>
       <c r="Q51" s="22" t="n"/>
       <c r="R51" s="22" t="n"/>
       <c r="S51" s="22" t="n"/>
@@ -7154,11 +7150,11 @@
     <row r="52" outlineLevel="1" ht="14" customHeight="1">
       <c r="A52" s="24" t="inlineStr">
         <is>
-          <t>8.2 Confirmación del pago</t>
+          <t>8.2 Guardar el método de pago</t>
         </is>
       </c>
       <c r="B52" s="22" t="n"/>
-      <c r="C52" s="22" t="n"/>
+      <c r="C52" s="28" t="n"/>
       <c r="D52" s="22" t="n"/>
       <c r="E52" s="22" t="n"/>
       <c r="F52" s="22" t="n"/>
@@ -7167,7 +7163,7 @@
       <c r="I52" s="22" t="n"/>
       <c r="J52" s="22" t="n"/>
       <c r="K52" s="22" t="n"/>
-      <c r="L52" s="28" t="n"/>
+      <c r="L52" s="22" t="n"/>
       <c r="M52" s="22" t="n"/>
       <c r="N52" s="22" t="n"/>
       <c r="O52" s="22" t="n"/>
@@ -7207,14 +7203,14 @@
       <c r="I53" s="22" t="n"/>
       <c r="J53" s="22" t="n"/>
       <c r="K53" s="22" t="n"/>
-      <c r="L53" s="21" t="n"/>
+      <c r="L53" s="22" t="n"/>
       <c r="M53" s="22" t="n"/>
       <c r="N53" s="22" t="n"/>
       <c r="O53" s="22" t="n"/>
       <c r="P53" s="22" t="n"/>
       <c r="Q53" s="22" t="n"/>
       <c r="R53" s="22" t="n"/>
-      <c r="S53" s="22" t="n"/>
+      <c r="S53" s="21" t="n"/>
       <c r="T53" s="22" t="n"/>
       <c r="U53" s="22" t="n"/>
       <c r="V53" s="22" t="n"/>
@@ -7238,24 +7234,24 @@
         </is>
       </c>
       <c r="B54" s="22" t="n"/>
-      <c r="C54" s="22" t="n"/>
+      <c r="C54" s="25" t="n"/>
       <c r="D54" s="22" t="n"/>
       <c r="E54" s="22" t="n"/>
       <c r="F54" s="22" t="n"/>
       <c r="G54" s="22" t="n"/>
       <c r="H54" s="22" t="n"/>
-      <c r="I54" s="25" t="n"/>
-      <c r="J54" s="25" t="n"/>
-      <c r="K54" s="25" t="n"/>
-      <c r="L54" s="25" t="n"/>
-      <c r="M54" s="25" t="n"/>
+      <c r="I54" s="22" t="n"/>
+      <c r="J54" s="22" t="n"/>
+      <c r="K54" s="22" t="n"/>
+      <c r="L54" s="22" t="n"/>
+      <c r="M54" s="22" t="n"/>
       <c r="N54" s="22" t="n"/>
       <c r="O54" s="22" t="n"/>
-      <c r="P54" s="22" t="n"/>
-      <c r="Q54" s="22" t="n"/>
-      <c r="R54" s="22" t="n"/>
-      <c r="S54" s="22" t="n"/>
-      <c r="T54" s="22" t="n"/>
+      <c r="P54" s="25" t="n"/>
+      <c r="Q54" s="25" t="n"/>
+      <c r="R54" s="25" t="n"/>
+      <c r="S54" s="25" t="n"/>
+      <c r="T54" s="25" t="n"/>
       <c r="U54" s="22" t="n"/>
       <c r="V54" s="22" t="n"/>
       <c r="W54" s="22" t="n"/>
@@ -7278,24 +7274,24 @@
         </is>
       </c>
       <c r="B55" s="22" t="n"/>
-      <c r="C55" s="22" t="n"/>
+      <c r="C55" s="26" t="n"/>
       <c r="D55" s="22" t="n"/>
       <c r="E55" s="22" t="n"/>
       <c r="F55" s="22" t="n"/>
       <c r="G55" s="22" t="n"/>
       <c r="H55" s="22" t="n"/>
-      <c r="I55" s="26" t="n"/>
-      <c r="J55" s="26" t="n"/>
-      <c r="K55" s="26" t="n"/>
-      <c r="L55" s="26" t="n"/>
-      <c r="M55" s="26" t="n"/>
+      <c r="I55" s="22" t="n"/>
+      <c r="J55" s="22" t="n"/>
+      <c r="K55" s="22" t="n"/>
+      <c r="L55" s="22" t="n"/>
+      <c r="M55" s="22" t="n"/>
       <c r="N55" s="22" t="n"/>
       <c r="O55" s="22" t="n"/>
-      <c r="P55" s="22" t="n"/>
-      <c r="Q55" s="22" t="n"/>
-      <c r="R55" s="22" t="n"/>
-      <c r="S55" s="22" t="n"/>
-      <c r="T55" s="22" t="n"/>
+      <c r="P55" s="26" t="n"/>
+      <c r="Q55" s="26" t="n"/>
+      <c r="R55" s="26" t="n"/>
+      <c r="S55" s="26" t="n"/>
+      <c r="T55" s="26" t="n"/>
       <c r="U55" s="22" t="n"/>
       <c r="V55" s="22" t="n"/>
       <c r="W55" s="22" t="n"/>
@@ -7320,7 +7316,7 @@
       <c r="B56" s="22" t="n"/>
       <c r="C56" s="22" t="n"/>
       <c r="D56" s="22" t="n"/>
-      <c r="E56" s="22" t="n"/>
+      <c r="E56" s="27" t="n"/>
       <c r="F56" s="22" t="n"/>
       <c r="G56" s="22" t="n"/>
       <c r="H56" s="22" t="n"/>
@@ -7329,15 +7325,15 @@
       <c r="K56" s="22" t="n"/>
       <c r="L56" s="22" t="n"/>
       <c r="M56" s="22" t="n"/>
-      <c r="N56" s="27" t="n"/>
-      <c r="O56" s="27" t="n"/>
+      <c r="N56" s="22" t="n"/>
+      <c r="O56" s="22" t="n"/>
       <c r="P56" s="22" t="n"/>
       <c r="Q56" s="22" t="n"/>
       <c r="R56" s="22" t="n"/>
       <c r="S56" s="22" t="n"/>
       <c r="T56" s="22" t="n"/>
-      <c r="U56" s="22" t="n"/>
-      <c r="V56" s="22" t="n"/>
+      <c r="U56" s="27" t="n"/>
+      <c r="V56" s="27" t="n"/>
       <c r="W56" s="22" t="n"/>
       <c r="X56" s="22" t="n"/>
       <c r="Y56" s="22" t="n"/>
@@ -7354,13 +7350,13 @@
     <row r="57" outlineLevel="1" ht="14" customHeight="1">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>9.1 Inicio del panel</t>
+          <t>9.1 Vista de admin descuadrada</t>
         </is>
       </c>
       <c r="B57" s="22" t="n"/>
       <c r="C57" s="22" t="n"/>
       <c r="D57" s="22" t="n"/>
-      <c r="E57" s="22" t="n"/>
+      <c r="E57" s="28" t="n"/>
       <c r="F57" s="22" t="n"/>
       <c r="G57" s="22" t="n"/>
       <c r="H57" s="22" t="n"/>
@@ -7369,7 +7365,7 @@
       <c r="K57" s="22" t="n"/>
       <c r="L57" s="22" t="n"/>
       <c r="M57" s="22" t="n"/>
-      <c r="N57" s="28" t="n"/>
+      <c r="N57" s="22" t="n"/>
       <c r="O57" s="22" t="n"/>
       <c r="P57" s="22" t="n"/>
       <c r="Q57" s="22" t="n"/>
@@ -7409,14 +7405,14 @@
       <c r="K58" s="22" t="n"/>
       <c r="L58" s="22" t="n"/>
       <c r="M58" s="22" t="n"/>
-      <c r="N58" s="21" t="n"/>
+      <c r="N58" s="22" t="n"/>
       <c r="O58" s="22" t="n"/>
       <c r="P58" s="22" t="n"/>
       <c r="Q58" s="22" t="n"/>
       <c r="R58" s="22" t="n"/>
       <c r="S58" s="22" t="n"/>
       <c r="T58" s="22" t="n"/>
-      <c r="U58" s="22" t="n"/>
+      <c r="U58" s="21" t="n"/>
       <c r="V58" s="22" t="n"/>
       <c r="W58" s="22" t="n"/>
       <c r="X58" s="22" t="n"/>
@@ -7449,14 +7445,14 @@
       <c r="K59" s="22" t="n"/>
       <c r="L59" s="22" t="n"/>
       <c r="M59" s="22" t="n"/>
-      <c r="N59" s="25" t="n"/>
+      <c r="N59" s="22" t="n"/>
       <c r="O59" s="22" t="n"/>
       <c r="P59" s="22" t="n"/>
       <c r="Q59" s="22" t="n"/>
       <c r="R59" s="22" t="n"/>
       <c r="S59" s="22" t="n"/>
       <c r="T59" s="22" t="n"/>
-      <c r="U59" s="22" t="n"/>
+      <c r="U59" s="25" t="n"/>
       <c r="V59" s="22" t="n"/>
       <c r="W59" s="22" t="n"/>
       <c r="X59" s="22" t="n"/>
@@ -7480,7 +7476,7 @@
       <c r="B60" s="22" t="n"/>
       <c r="C60" s="22" t="n"/>
       <c r="D60" s="22" t="n"/>
-      <c r="E60" s="22" t="n"/>
+      <c r="E60" s="26" t="n"/>
       <c r="F60" s="22" t="n"/>
       <c r="G60" s="22" t="n"/>
       <c r="H60" s="22" t="n"/>
@@ -7489,15 +7485,15 @@
       <c r="K60" s="22" t="n"/>
       <c r="L60" s="22" t="n"/>
       <c r="M60" s="22" t="n"/>
-      <c r="N60" s="26" t="n"/>
-      <c r="O60" s="26" t="n"/>
+      <c r="N60" s="22" t="n"/>
+      <c r="O60" s="22" t="n"/>
       <c r="P60" s="22" t="n"/>
       <c r="Q60" s="22" t="n"/>
       <c r="R60" s="22" t="n"/>
       <c r="S60" s="22" t="n"/>
       <c r="T60" s="22" t="n"/>
-      <c r="U60" s="22" t="n"/>
-      <c r="V60" s="22" t="n"/>
+      <c r="U60" s="26" t="n"/>
+      <c r="V60" s="26" t="n"/>
       <c r="W60" s="22" t="n"/>
       <c r="X60" s="22" t="n"/>
       <c r="Y60" s="22" t="n"/>
@@ -7520,7 +7516,7 @@
       <c r="B61" s="22" t="n"/>
       <c r="C61" s="22" t="n"/>
       <c r="D61" s="22" t="n"/>
-      <c r="E61" s="22" t="n"/>
+      <c r="E61" s="27" t="n"/>
       <c r="F61" s="22" t="n"/>
       <c r="G61" s="22" t="n"/>
       <c r="H61" s="22" t="n"/>
@@ -7529,15 +7525,15 @@
       <c r="K61" s="22" t="n"/>
       <c r="L61" s="22" t="n"/>
       <c r="M61" s="22" t="n"/>
-      <c r="N61" s="27" t="n"/>
-      <c r="O61" s="27" t="n"/>
+      <c r="N61" s="22" t="n"/>
+      <c r="O61" s="22" t="n"/>
       <c r="P61" s="22" t="n"/>
       <c r="Q61" s="22" t="n"/>
       <c r="R61" s="22" t="n"/>
       <c r="S61" s="22" t="n"/>
       <c r="T61" s="22" t="n"/>
-      <c r="U61" s="22" t="n"/>
-      <c r="V61" s="22" t="n"/>
+      <c r="U61" s="27" t="n"/>
+      <c r="V61" s="27" t="n"/>
       <c r="W61" s="22" t="n"/>
       <c r="X61" s="22" t="n"/>
       <c r="Y61" s="22" t="n"/>
@@ -7559,7 +7555,7 @@
       </c>
       <c r="B62" s="22" t="n"/>
       <c r="C62" s="22" t="n"/>
-      <c r="D62" s="22" t="n"/>
+      <c r="D62" s="28" t="n"/>
       <c r="E62" s="22" t="n"/>
       <c r="F62" s="22" t="n"/>
       <c r="G62" s="22" t="n"/>
@@ -7571,17 +7567,17 @@
       <c r="M62" s="22" t="n"/>
       <c r="N62" s="22" t="n"/>
       <c r="O62" s="22" t="n"/>
-      <c r="P62" s="28" t="n"/>
-      <c r="Q62" s="28" t="n"/>
-      <c r="R62" s="28" t="n"/>
-      <c r="S62" s="28" t="n"/>
+      <c r="P62" s="22" t="n"/>
+      <c r="Q62" s="22" t="n"/>
+      <c r="R62" s="22" t="n"/>
+      <c r="S62" s="22" t="n"/>
       <c r="T62" s="22" t="n"/>
       <c r="U62" s="22" t="n"/>
       <c r="V62" s="22" t="n"/>
-      <c r="W62" s="22" t="n"/>
-      <c r="X62" s="22" t="n"/>
-      <c r="Y62" s="22" t="n"/>
-      <c r="Z62" s="22" t="n"/>
+      <c r="W62" s="28" t="n"/>
+      <c r="X62" s="28" t="n"/>
+      <c r="Y62" s="28" t="n"/>
+      <c r="Z62" s="28" t="n"/>
       <c r="AA62" s="22" t="n"/>
       <c r="AB62" s="22" t="n"/>
       <c r="AC62" s="22" t="n"/>
@@ -7611,14 +7607,14 @@
       <c r="M63" s="22" t="n"/>
       <c r="N63" s="22" t="n"/>
       <c r="O63" s="22" t="n"/>
-      <c r="P63" s="21" t="n"/>
+      <c r="P63" s="22" t="n"/>
       <c r="Q63" s="22" t="n"/>
       <c r="R63" s="22" t="n"/>
       <c r="S63" s="22" t="n"/>
       <c r="T63" s="22" t="n"/>
       <c r="U63" s="22" t="n"/>
       <c r="V63" s="22" t="n"/>
-      <c r="W63" s="22" t="n"/>
+      <c r="W63" s="21" t="n"/>
       <c r="X63" s="22" t="n"/>
       <c r="Y63" s="22" t="n"/>
       <c r="Z63" s="22" t="n"/>
@@ -7651,14 +7647,14 @@
       <c r="M64" s="22" t="n"/>
       <c r="N64" s="22" t="n"/>
       <c r="O64" s="22" t="n"/>
-      <c r="P64" s="25" t="n"/>
+      <c r="P64" s="22" t="n"/>
       <c r="Q64" s="22" t="n"/>
       <c r="R64" s="22" t="n"/>
       <c r="S64" s="22" t="n"/>
       <c r="T64" s="22" t="n"/>
       <c r="U64" s="22" t="n"/>
       <c r="V64" s="22" t="n"/>
-      <c r="W64" s="22" t="n"/>
+      <c r="W64" s="25" t="n"/>
       <c r="X64" s="22" t="n"/>
       <c r="Y64" s="22" t="n"/>
       <c r="Z64" s="22" t="n"/>
@@ -7674,12 +7670,12 @@
     <row r="65" outlineLevel="1" ht="14" customHeight="1">
       <c r="A65" s="24" t="inlineStr">
         <is>
-          <t>10.3 Edición de datos</t>
+          <t>10.3 Impersonalidad: usuario1</t>
         </is>
       </c>
       <c r="B65" s="22" t="n"/>
       <c r="C65" s="22" t="n"/>
-      <c r="D65" s="22" t="n"/>
+      <c r="D65" s="26" t="n"/>
       <c r="E65" s="22" t="n"/>
       <c r="F65" s="22" t="n"/>
       <c r="G65" s="22" t="n"/>
@@ -7691,7 +7687,7 @@
       <c r="M65" s="22" t="n"/>
       <c r="N65" s="22" t="n"/>
       <c r="O65" s="22" t="n"/>
-      <c r="P65" s="26" t="n"/>
+      <c r="P65" s="22" t="n"/>
       <c r="Q65" s="22" t="n"/>
       <c r="R65" s="22" t="n"/>
       <c r="S65" s="22" t="n"/>
@@ -7719,7 +7715,7 @@
       </c>
       <c r="B66" s="22" t="n"/>
       <c r="C66" s="22" t="n"/>
-      <c r="D66" s="22" t="n"/>
+      <c r="D66" s="27" t="n"/>
       <c r="E66" s="22" t="n"/>
       <c r="F66" s="22" t="n"/>
       <c r="G66" s="22" t="n"/>
@@ -7731,17 +7727,17 @@
       <c r="M66" s="22" t="n"/>
       <c r="N66" s="22" t="n"/>
       <c r="O66" s="22" t="n"/>
-      <c r="P66" s="27" t="n"/>
-      <c r="Q66" s="27" t="n"/>
-      <c r="R66" s="27" t="n"/>
-      <c r="S66" s="27" t="n"/>
+      <c r="P66" s="22" t="n"/>
+      <c r="Q66" s="22" t="n"/>
+      <c r="R66" s="22" t="n"/>
+      <c r="S66" s="22" t="n"/>
       <c r="T66" s="22" t="n"/>
       <c r="U66" s="22" t="n"/>
       <c r="V66" s="22" t="n"/>
-      <c r="W66" s="22" t="n"/>
-      <c r="X66" s="22" t="n"/>
-      <c r="Y66" s="22" t="n"/>
-      <c r="Z66" s="22" t="n"/>
+      <c r="W66" s="27" t="n"/>
+      <c r="X66" s="27" t="n"/>
+      <c r="Y66" s="27" t="n"/>
+      <c r="Z66" s="27" t="n"/>
       <c r="AA66" s="22" t="n"/>
       <c r="AB66" s="22" t="n"/>
       <c r="AC66" s="22" t="n"/>
@@ -7759,7 +7755,7 @@
       </c>
       <c r="B67" s="22" t="n"/>
       <c r="C67" s="22" t="n"/>
-      <c r="D67" s="22" t="n"/>
+      <c r="D67" s="28" t="n"/>
       <c r="E67" s="22" t="n"/>
       <c r="F67" s="22" t="n"/>
       <c r="G67" s="22" t="n"/>
@@ -7771,17 +7767,17 @@
       <c r="M67" s="22" t="n"/>
       <c r="N67" s="22" t="n"/>
       <c r="O67" s="22" t="n"/>
-      <c r="P67" s="28" t="n"/>
-      <c r="Q67" s="28" t="n"/>
-      <c r="R67" s="28" t="n"/>
-      <c r="S67" s="28" t="n"/>
+      <c r="P67" s="22" t="n"/>
+      <c r="Q67" s="22" t="n"/>
+      <c r="R67" s="22" t="n"/>
+      <c r="S67" s="22" t="n"/>
       <c r="T67" s="22" t="n"/>
       <c r="U67" s="22" t="n"/>
       <c r="V67" s="22" t="n"/>
-      <c r="W67" s="22" t="n"/>
-      <c r="X67" s="22" t="n"/>
-      <c r="Y67" s="22" t="n"/>
-      <c r="Z67" s="22" t="n"/>
+      <c r="W67" s="28" t="n"/>
+      <c r="X67" s="28" t="n"/>
+      <c r="Y67" s="28" t="n"/>
+      <c r="Z67" s="28" t="n"/>
       <c r="AA67" s="22" t="n"/>
       <c r="AB67" s="22" t="n"/>
       <c r="AC67" s="22" t="n"/>
@@ -7794,14 +7790,14 @@
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="20" t="inlineStr">
         <is>
-          <t>11. Monitores y solicitudes</t>
+          <t>11. Monitores y reportes</t>
         </is>
       </c>
       <c r="B68" s="22" t="n"/>
       <c r="C68" s="22" t="n"/>
-      <c r="D68" s="22" t="n"/>
+      <c r="D68" s="21" t="n"/>
       <c r="E68" s="22" t="n"/>
-      <c r="F68" s="22" t="n"/>
+      <c r="F68" s="21" t="n"/>
       <c r="G68" s="22" t="n"/>
       <c r="H68" s="22" t="n"/>
       <c r="I68" s="22" t="n"/>
@@ -7815,16 +7811,16 @@
       <c r="Q68" s="22" t="n"/>
       <c r="R68" s="22" t="n"/>
       <c r="S68" s="22" t="n"/>
-      <c r="T68" s="21" t="n"/>
-      <c r="U68" s="21" t="n"/>
-      <c r="V68" s="21" t="n"/>
+      <c r="T68" s="22" t="n"/>
+      <c r="U68" s="22" t="n"/>
+      <c r="V68" s="22" t="n"/>
       <c r="W68" s="22" t="n"/>
       <c r="X68" s="22" t="n"/>
       <c r="Y68" s="22" t="n"/>
       <c r="Z68" s="22" t="n"/>
-      <c r="AA68" s="22" t="n"/>
-      <c r="AB68" s="22" t="n"/>
-      <c r="AC68" s="22" t="n"/>
+      <c r="AA68" s="21" t="n"/>
+      <c r="AB68" s="21" t="n"/>
+      <c r="AC68" s="21" t="n"/>
       <c r="AD68" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -7834,12 +7830,12 @@
     <row r="69" outlineLevel="1" ht="14" customHeight="1">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t>11.1 Alta de monitores</t>
+          <t>11.1 Impersonalidad: monitor1</t>
         </is>
       </c>
       <c r="B69" s="22" t="n"/>
       <c r="C69" s="22" t="n"/>
-      <c r="D69" s="22" t="n"/>
+      <c r="D69" s="25" t="n"/>
       <c r="E69" s="22" t="n"/>
       <c r="F69" s="22" t="n"/>
       <c r="G69" s="22" t="n"/>
@@ -7855,7 +7851,7 @@
       <c r="Q69" s="22" t="n"/>
       <c r="R69" s="22" t="n"/>
       <c r="S69" s="22" t="n"/>
-      <c r="T69" s="25" t="n"/>
+      <c r="T69" s="22" t="n"/>
       <c r="U69" s="22" t="n"/>
       <c r="V69" s="22" t="n"/>
       <c r="W69" s="22" t="n"/>
@@ -7874,14 +7870,14 @@
     <row r="70" outlineLevel="1" ht="14" customHeight="1">
       <c r="A70" s="24" t="inlineStr">
         <is>
-          <t>11.2 Solicitudes de clase</t>
+          <t>11.2 De solicitudes a reportes</t>
         </is>
       </c>
       <c r="B70" s="22" t="n"/>
       <c r="C70" s="22" t="n"/>
       <c r="D70" s="22" t="n"/>
       <c r="E70" s="22" t="n"/>
-      <c r="F70" s="22" t="n"/>
+      <c r="F70" s="26" t="n"/>
       <c r="G70" s="22" t="n"/>
       <c r="H70" s="22" t="n"/>
       <c r="I70" s="22" t="n"/>
@@ -7896,7 +7892,7 @@
       <c r="R70" s="22" t="n"/>
       <c r="S70" s="22" t="n"/>
       <c r="T70" s="22" t="n"/>
-      <c r="U70" s="26" t="n"/>
+      <c r="U70" s="22" t="n"/>
       <c r="V70" s="22" t="n"/>
       <c r="W70" s="22" t="n"/>
       <c r="X70" s="22" t="n"/>
@@ -7936,14 +7932,14 @@
       <c r="R71" s="22" t="n"/>
       <c r="S71" s="22" t="n"/>
       <c r="T71" s="22" t="n"/>
-      <c r="U71" s="27" t="n"/>
+      <c r="U71" s="22" t="n"/>
       <c r="V71" s="22" t="n"/>
       <c r="W71" s="22" t="n"/>
       <c r="X71" s="22" t="n"/>
       <c r="Y71" s="22" t="n"/>
       <c r="Z71" s="22" t="n"/>
       <c r="AA71" s="22" t="n"/>
-      <c r="AB71" s="22" t="n"/>
+      <c r="AB71" s="27" t="n"/>
       <c r="AC71" s="22" t="n"/>
       <c r="AD71" s="30" t="inlineStr">
         <is>
@@ -7959,9 +7955,9 @@
       </c>
       <c r="B72" s="22" t="n"/>
       <c r="C72" s="22" t="n"/>
-      <c r="D72" s="22" t="n"/>
+      <c r="D72" s="28" t="n"/>
       <c r="E72" s="22" t="n"/>
-      <c r="F72" s="22" t="n"/>
+      <c r="F72" s="28" t="n"/>
       <c r="G72" s="22" t="n"/>
       <c r="H72" s="22" t="n"/>
       <c r="I72" s="22" t="n"/>
@@ -7975,16 +7971,16 @@
       <c r="Q72" s="22" t="n"/>
       <c r="R72" s="22" t="n"/>
       <c r="S72" s="22" t="n"/>
-      <c r="T72" s="28" t="n"/>
-      <c r="U72" s="28" t="n"/>
-      <c r="V72" s="28" t="n"/>
+      <c r="T72" s="22" t="n"/>
+      <c r="U72" s="22" t="n"/>
+      <c r="V72" s="22" t="n"/>
       <c r="W72" s="22" t="n"/>
       <c r="X72" s="22" t="n"/>
       <c r="Y72" s="22" t="n"/>
       <c r="Z72" s="22" t="n"/>
-      <c r="AA72" s="22" t="n"/>
-      <c r="AB72" s="22" t="n"/>
-      <c r="AC72" s="22" t="n"/>
+      <c r="AA72" s="28" t="n"/>
+      <c r="AB72" s="28" t="n"/>
+      <c r="AC72" s="28" t="n"/>
       <c r="AD72" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -7999,9 +7995,9 @@
       </c>
       <c r="B73" s="22" t="n"/>
       <c r="C73" s="22" t="n"/>
-      <c r="D73" s="22" t="n"/>
+      <c r="D73" s="21" t="n"/>
       <c r="E73" s="22" t="n"/>
-      <c r="F73" s="22" t="n"/>
+      <c r="F73" s="21" t="n"/>
       <c r="G73" s="22" t="n"/>
       <c r="H73" s="22" t="n"/>
       <c r="I73" s="22" t="n"/>
@@ -8015,16 +8011,16 @@
       <c r="Q73" s="22" t="n"/>
       <c r="R73" s="22" t="n"/>
       <c r="S73" s="22" t="n"/>
-      <c r="T73" s="21" t="n"/>
-      <c r="U73" s="21" t="n"/>
-      <c r="V73" s="21" t="n"/>
+      <c r="T73" s="22" t="n"/>
+      <c r="U73" s="22" t="n"/>
+      <c r="V73" s="22" t="n"/>
       <c r="W73" s="22" t="n"/>
       <c r="X73" s="22" t="n"/>
       <c r="Y73" s="22" t="n"/>
       <c r="Z73" s="22" t="n"/>
-      <c r="AA73" s="22" t="n"/>
-      <c r="AB73" s="22" t="n"/>
-      <c r="AC73" s="22" t="n"/>
+      <c r="AA73" s="21" t="n"/>
+      <c r="AB73" s="21" t="n"/>
+      <c r="AC73" s="21" t="n"/>
       <c r="AD73" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -8041,7 +8037,7 @@
       <c r="C74" s="22" t="n"/>
       <c r="D74" s="22" t="n"/>
       <c r="E74" s="22" t="n"/>
-      <c r="F74" s="22" t="n"/>
+      <c r="F74" s="25" t="n"/>
       <c r="G74" s="22" t="n"/>
       <c r="H74" s="22" t="n"/>
       <c r="I74" s="22" t="n"/>
@@ -8058,10 +8054,10 @@
       <c r="T74" s="22" t="n"/>
       <c r="U74" s="22" t="n"/>
       <c r="V74" s="22" t="n"/>
-      <c r="W74" s="25" t="n"/>
-      <c r="X74" s="25" t="n"/>
-      <c r="Y74" s="25" t="n"/>
-      <c r="Z74" s="25" t="n"/>
+      <c r="W74" s="22" t="n"/>
+      <c r="X74" s="22" t="n"/>
+      <c r="Y74" s="22" t="n"/>
+      <c r="Z74" s="22" t="n"/>
       <c r="AA74" s="22" t="n"/>
       <c r="AB74" s="22" t="n"/>
       <c r="AC74" s="22" t="n"/>
@@ -8074,14 +8070,14 @@
     <row r="75" outlineLevel="1" ht="14" customHeight="1">
       <c r="A75" s="24" t="inlineStr">
         <is>
-          <t>12.1 Ficha de salas</t>
+          <t>12.1 Colores de salas y actividades</t>
         </is>
       </c>
       <c r="B75" s="22" t="n"/>
       <c r="C75" s="22" t="n"/>
       <c r="D75" s="22" t="n"/>
       <c r="E75" s="22" t="n"/>
-      <c r="F75" s="22" t="n"/>
+      <c r="F75" s="26" t="n"/>
       <c r="G75" s="22" t="n"/>
       <c r="H75" s="22" t="n"/>
       <c r="I75" s="22" t="n"/>
@@ -8098,7 +8094,7 @@
       <c r="T75" s="22" t="n"/>
       <c r="U75" s="22" t="n"/>
       <c r="V75" s="22" t="n"/>
-      <c r="W75" s="26" t="n"/>
+      <c r="W75" s="22" t="n"/>
       <c r="X75" s="22" t="n"/>
       <c r="Y75" s="22" t="n"/>
       <c r="Z75" s="22" t="n"/>
@@ -8138,7 +8134,7 @@
       <c r="T76" s="22" t="n"/>
       <c r="U76" s="22" t="n"/>
       <c r="V76" s="22" t="n"/>
-      <c r="W76" s="27" t="n"/>
+      <c r="W76" s="22" t="n"/>
       <c r="X76" s="22" t="n"/>
       <c r="Y76" s="22" t="n"/>
       <c r="Z76" s="22" t="n"/>
@@ -8178,7 +8174,7 @@
       <c r="T77" s="22" t="n"/>
       <c r="U77" s="22" t="n"/>
       <c r="V77" s="22" t="n"/>
-      <c r="W77" s="28" t="n"/>
+      <c r="W77" s="22" t="n"/>
       <c r="X77" s="22" t="n"/>
       <c r="Y77" s="22" t="n"/>
       <c r="Z77" s="22" t="n"/>
@@ -8201,7 +8197,7 @@
       <c r="C78" s="22" t="n"/>
       <c r="D78" s="22" t="n"/>
       <c r="E78" s="22" t="n"/>
-      <c r="F78" s="22" t="n"/>
+      <c r="F78" s="21" t="n"/>
       <c r="G78" s="22" t="n"/>
       <c r="H78" s="22" t="n"/>
       <c r="I78" s="22" t="n"/>
@@ -8218,10 +8214,10 @@
       <c r="T78" s="22" t="n"/>
       <c r="U78" s="22" t="n"/>
       <c r="V78" s="22" t="n"/>
-      <c r="W78" s="21" t="n"/>
-      <c r="X78" s="21" t="n"/>
-      <c r="Y78" s="21" t="n"/>
-      <c r="Z78" s="21" t="n"/>
+      <c r="W78" s="22" t="n"/>
+      <c r="X78" s="22" t="n"/>
+      <c r="Y78" s="22" t="n"/>
+      <c r="Z78" s="22" t="n"/>
       <c r="AA78" s="22" t="n"/>
       <c r="AB78" s="22" t="n"/>
       <c r="AC78" s="22" t="n"/>
@@ -8241,7 +8237,7 @@
       <c r="C79" s="22" t="n"/>
       <c r="D79" s="22" t="n"/>
       <c r="E79" s="22" t="n"/>
-      <c r="F79" s="22" t="n"/>
+      <c r="F79" s="25" t="n"/>
       <c r="G79" s="22" t="n"/>
       <c r="H79" s="22" t="n"/>
       <c r="I79" s="22" t="n"/>
@@ -8258,10 +8254,10 @@
       <c r="T79" s="22" t="n"/>
       <c r="U79" s="22" t="n"/>
       <c r="V79" s="22" t="n"/>
-      <c r="W79" s="25" t="n"/>
-      <c r="X79" s="25" t="n"/>
-      <c r="Y79" s="25" t="n"/>
-      <c r="Z79" s="25" t="n"/>
+      <c r="W79" s="22" t="n"/>
+      <c r="X79" s="22" t="n"/>
+      <c r="Y79" s="22" t="n"/>
+      <c r="Z79" s="22" t="n"/>
       <c r="AA79" s="22" t="n"/>
       <c r="AB79" s="22" t="n"/>
       <c r="AC79" s="22" t="n"/>
@@ -8302,9 +8298,9 @@
       <c r="X80" s="22" t="n"/>
       <c r="Y80" s="22" t="n"/>
       <c r="Z80" s="22" t="n"/>
-      <c r="AA80" s="26" t="n"/>
-      <c r="AB80" s="26" t="n"/>
-      <c r="AC80" s="26" t="n"/>
+      <c r="AA80" s="22" t="n"/>
+      <c r="AB80" s="22" t="n"/>
+      <c r="AC80" s="22" t="n"/>
       <c r="AD80" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -8342,7 +8338,7 @@
       <c r="X81" s="22" t="n"/>
       <c r="Y81" s="22" t="n"/>
       <c r="Z81" s="22" t="n"/>
-      <c r="AA81" s="27" t="n"/>
+      <c r="AA81" s="22" t="n"/>
       <c r="AB81" s="22" t="n"/>
       <c r="AC81" s="22" t="n"/>
       <c r="AD81" s="30" t="inlineStr">
@@ -8383,7 +8379,7 @@
       <c r="Y82" s="22" t="n"/>
       <c r="Z82" s="22" t="n"/>
       <c r="AA82" s="22" t="n"/>
-      <c r="AB82" s="28" t="n"/>
+      <c r="AB82" s="22" t="n"/>
       <c r="AC82" s="22" t="n"/>
       <c r="AD82" s="30" t="inlineStr">
         <is>
@@ -8423,7 +8419,7 @@
       <c r="Y83" s="22" t="n"/>
       <c r="Z83" s="22" t="n"/>
       <c r="AA83" s="22" t="n"/>
-      <c r="AB83" s="21" t="n"/>
+      <c r="AB83" s="22" t="n"/>
       <c r="AC83" s="22" t="n"/>
       <c r="AD83" s="30" t="inlineStr">
         <is>
@@ -8462,9 +8458,9 @@
       <c r="X84" s="22" t="n"/>
       <c r="Y84" s="22" t="n"/>
       <c r="Z84" s="22" t="n"/>
-      <c r="AA84" s="25" t="n"/>
-      <c r="AB84" s="25" t="n"/>
-      <c r="AC84" s="25" t="n"/>
+      <c r="AA84" s="22" t="n"/>
+      <c r="AB84" s="22" t="n"/>
+      <c r="AC84" s="22" t="n"/>
       <c r="AD84" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -8502,9 +8498,9 @@
       <c r="X85" s="22" t="n"/>
       <c r="Y85" s="22" t="n"/>
       <c r="Z85" s="22" t="n"/>
-      <c r="AA85" s="26" t="n"/>
-      <c r="AB85" s="26" t="n"/>
-      <c r="AC85" s="26" t="n"/>
+      <c r="AA85" s="22" t="n"/>
+      <c r="AB85" s="22" t="n"/>
+      <c r="AC85" s="22" t="n"/>
       <c r="AD85" s="30" t="inlineStr">
         <is>
           <t>sin iniciar</t>
@@ -8825,9 +8821,9 @@
       <c r="AA93" s="22" t="n"/>
       <c r="AB93" s="22" t="n"/>
       <c r="AC93" s="22" t="n"/>
-      <c r="AD93" s="29" t="inlineStr">
-        <is>
-          <t>en curso</t>
+      <c r="AD93" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -8865,9 +8861,9 @@
       <c r="AA94" s="22" t="n"/>
       <c r="AB94" s="22" t="n"/>
       <c r="AC94" s="22" t="n"/>
-      <c r="AD94" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="AD94" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -9125,12 +9121,12 @@
     <mergeCell ref="I5:O5"/>
     <mergeCell ref="P5:V5"/>
     <mergeCell ref="W4:AC4"/>
+    <mergeCell ref="AD4:AD7"/>
+    <mergeCell ref="B4:H4"/>
     <mergeCell ref="W5:AC5"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="AD4:AD7"/>
     <mergeCell ref="P4:V4"/>
+    <mergeCell ref="A2:AD2"/>
     <mergeCell ref="I4:O4"/>
-    <mergeCell ref="A2:AD2"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
@@ -9148,7 +9144,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W101"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="3.7" customWidth="1" min="2" max="2"/>
@@ -10093,9 +10089,9 @@
       <c r="T26" s="22" t="n"/>
       <c r="U26" s="22" t="n"/>
       <c r="V26" s="22" t="n"/>
-      <c r="W26" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W26" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10168,7 +10164,7 @@
     <row r="29" outlineLevel="1" ht="14" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>4.3 Baja y reactivación</t>
+          <t>4.3 Baja: al redirigir se pierde la sesión</t>
         </is>
       </c>
       <c r="B29" s="22" t="n"/>
@@ -10192,9 +10188,9 @@
       <c r="T29" s="22" t="n"/>
       <c r="U29" s="22" t="n"/>
       <c r="V29" s="22" t="n"/>
-      <c r="W29" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W29" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10225,9 +10221,9 @@
       <c r="T30" s="22" t="n"/>
       <c r="U30" s="22" t="n"/>
       <c r="V30" s="22" t="n"/>
-      <c r="W30" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W30" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10258,9 +10254,9 @@
       <c r="T31" s="22" t="n"/>
       <c r="U31" s="22" t="n"/>
       <c r="V31" s="22" t="n"/>
-      <c r="W31" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W31" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10296,7 @@
     <row r="33" outlineLevel="1" ht="14" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>5.1 Listado de actividades</t>
+          <t>5.1 Listado descuadrado</t>
         </is>
       </c>
       <c r="B33" s="22" t="n"/>
@@ -10324,16 +10320,16 @@
       <c r="T33" s="22" t="n"/>
       <c r="U33" s="22" t="n"/>
       <c r="V33" s="22" t="n"/>
-      <c r="W33" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W33" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
     <row r="34" outlineLevel="1" ht="14" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>5.2 Horario y avisos → inscritos</t>
+          <t>5.2 Horario con uniformidad</t>
         </is>
       </c>
       <c r="B34" s="22" t="n"/>
@@ -10357,9 +10353,9 @@
       <c r="T34" s="22" t="n"/>
       <c r="U34" s="22" t="n"/>
       <c r="V34" s="22" t="n"/>
-      <c r="W34" s="23" t="inlineStr">
-        <is>
-          <t>completado</t>
+      <c r="W34" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -10390,9 +10386,9 @@
       <c r="T35" s="22" t="n"/>
       <c r="U35" s="22" t="n"/>
       <c r="V35" s="22" t="n"/>
-      <c r="W35" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W35" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10687,9 +10683,9 @@
       <c r="T44" s="22" t="n"/>
       <c r="U44" s="22" t="n"/>
       <c r="V44" s="22" t="n"/>
-      <c r="W44" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W44" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10720,9 +10716,9 @@
       <c r="T45" s="22" t="n"/>
       <c r="U45" s="22" t="n"/>
       <c r="V45" s="22" t="n"/>
-      <c r="W45" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W45" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10753,9 +10749,9 @@
       <c r="T46" s="22" t="n"/>
       <c r="U46" s="22" t="n"/>
       <c r="V46" s="22" t="n"/>
-      <c r="W46" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W46" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10786,9 +10782,9 @@
       <c r="T47" s="22" t="n"/>
       <c r="U47" s="22" t="n"/>
       <c r="V47" s="22" t="n"/>
-      <c r="W47" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W47" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10819,9 +10815,9 @@
       <c r="T48" s="22" t="n"/>
       <c r="U48" s="22" t="n"/>
       <c r="V48" s="22" t="n"/>
-      <c r="W48" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W48" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10852,9 +10848,9 @@
       <c r="T49" s="22" t="n"/>
       <c r="U49" s="22" t="n"/>
       <c r="V49" s="22" t="n"/>
-      <c r="W49" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W49" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -10927,7 +10923,7 @@
     <row r="52" outlineLevel="1" ht="14" customHeight="1">
       <c r="A52" s="24" t="inlineStr">
         <is>
-          <t>8.2 Confirmación del pago</t>
+          <t>8.2 Guardar el método de pago</t>
         </is>
       </c>
       <c r="B52" s="22" t="n"/>
@@ -11092,7 +11088,7 @@
     <row r="57" outlineLevel="1" ht="14" customHeight="1">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>9.1 Inicio del panel</t>
+          <t>9.1 Vista de admin descuadrada</t>
         </is>
       </c>
       <c r="B57" s="22" t="n"/>
@@ -11356,7 +11352,7 @@
     <row r="65" outlineLevel="1" ht="14" customHeight="1">
       <c r="A65" s="24" t="inlineStr">
         <is>
-          <t>10.3 Edición de datos</t>
+          <t>10.3 Impersonalidad: usuario1</t>
         </is>
       </c>
       <c r="B65" s="22" t="n"/>
@@ -11455,7 +11451,7 @@
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="20" t="inlineStr">
         <is>
-          <t>11. Monitores y solicitudes</t>
+          <t>11. Monitores y reportes</t>
         </is>
       </c>
       <c r="B68" s="22" t="n"/>
@@ -11488,7 +11484,7 @@
     <row r="69" outlineLevel="1" ht="14" customHeight="1">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t>11.1 Alta de monitores</t>
+          <t>11.1 Impersonalidad: monitor1</t>
         </is>
       </c>
       <c r="B69" s="22" t="n"/>
@@ -11521,7 +11517,7 @@
     <row r="70" outlineLevel="1" ht="14" customHeight="1">
       <c r="A70" s="24" t="inlineStr">
         <is>
-          <t>11.2 Solicitudes de clase</t>
+          <t>11.2 De solicitudes a reportes</t>
         </is>
       </c>
       <c r="B70" s="22" t="n"/>
@@ -11656,10 +11652,10 @@
           <t>12. Salas y materiales</t>
         </is>
       </c>
-      <c r="B74" s="22" t="n"/>
-      <c r="C74" s="22" t="n"/>
-      <c r="D74" s="22" t="n"/>
-      <c r="E74" s="22" t="n"/>
+      <c r="B74" s="25" t="n"/>
+      <c r="C74" s="25" t="n"/>
+      <c r="D74" s="25" t="n"/>
+      <c r="E74" s="25" t="n"/>
       <c r="F74" s="22" t="n"/>
       <c r="G74" s="22" t="n"/>
       <c r="H74" s="22" t="n"/>
@@ -11686,7 +11682,7 @@
     <row r="75" outlineLevel="1" ht="14" customHeight="1">
       <c r="A75" s="24" t="inlineStr">
         <is>
-          <t>12.1 Ficha de salas</t>
+          <t>12.1 Colores de salas y actividades</t>
         </is>
       </c>
       <c r="B75" s="22" t="n"/>
@@ -11722,7 +11718,7 @@
           <t>12.2 Inventario de materiales</t>
         </is>
       </c>
-      <c r="B76" s="22" t="n"/>
+      <c r="B76" s="27" t="n"/>
       <c r="C76" s="22" t="n"/>
       <c r="D76" s="22" t="n"/>
       <c r="E76" s="22" t="n"/>
@@ -11755,7 +11751,7 @@
           <t>12.3 Alta y edición</t>
         </is>
       </c>
-      <c r="B77" s="22" t="n"/>
+      <c r="B77" s="28" t="n"/>
       <c r="C77" s="22" t="n"/>
       <c r="D77" s="22" t="n"/>
       <c r="E77" s="22" t="n"/>
@@ -11788,10 +11784,10 @@
           <t>12.4 Testeo</t>
         </is>
       </c>
-      <c r="B78" s="22" t="n"/>
-      <c r="C78" s="22" t="n"/>
-      <c r="D78" s="22" t="n"/>
-      <c r="E78" s="22" t="n"/>
+      <c r="B78" s="21" t="n"/>
+      <c r="C78" s="21" t="n"/>
+      <c r="D78" s="21" t="n"/>
+      <c r="E78" s="21" t="n"/>
       <c r="F78" s="22" t="n"/>
       <c r="G78" s="22" t="n"/>
       <c r="H78" s="22" t="n"/>
@@ -11821,10 +11817,10 @@
           <t>12.5 Documentación</t>
         </is>
       </c>
-      <c r="B79" s="22" t="n"/>
-      <c r="C79" s="22" t="n"/>
-      <c r="D79" s="22" t="n"/>
-      <c r="E79" s="22" t="n"/>
+      <c r="B79" s="25" t="n"/>
+      <c r="C79" s="25" t="n"/>
+      <c r="D79" s="25" t="n"/>
+      <c r="E79" s="25" t="n"/>
       <c r="F79" s="22" t="n"/>
       <c r="G79" s="22" t="n"/>
       <c r="H79" s="22" t="n"/>
@@ -11858,9 +11854,9 @@
       <c r="C80" s="22" t="n"/>
       <c r="D80" s="22" t="n"/>
       <c r="E80" s="22" t="n"/>
-      <c r="F80" s="22" t="n"/>
-      <c r="G80" s="22" t="n"/>
-      <c r="H80" s="22" t="n"/>
+      <c r="F80" s="26" t="n"/>
+      <c r="G80" s="26" t="n"/>
+      <c r="H80" s="26" t="n"/>
       <c r="I80" s="22" t="n"/>
       <c r="J80" s="22" t="n"/>
       <c r="K80" s="22" t="n"/>
@@ -11891,7 +11887,7 @@
       <c r="C81" s="22" t="n"/>
       <c r="D81" s="22" t="n"/>
       <c r="E81" s="22" t="n"/>
-      <c r="F81" s="22" t="n"/>
+      <c r="F81" s="27" t="n"/>
       <c r="G81" s="22" t="n"/>
       <c r="H81" s="22" t="n"/>
       <c r="I81" s="22" t="n"/>
@@ -11925,7 +11921,7 @@
       <c r="D82" s="22" t="n"/>
       <c r="E82" s="22" t="n"/>
       <c r="F82" s="22" t="n"/>
-      <c r="G82" s="22" t="n"/>
+      <c r="G82" s="28" t="n"/>
       <c r="H82" s="22" t="n"/>
       <c r="I82" s="22" t="n"/>
       <c r="J82" s="22" t="n"/>
@@ -11958,7 +11954,7 @@
       <c r="D83" s="22" t="n"/>
       <c r="E83" s="22" t="n"/>
       <c r="F83" s="22" t="n"/>
-      <c r="G83" s="22" t="n"/>
+      <c r="G83" s="21" t="n"/>
       <c r="H83" s="22" t="n"/>
       <c r="I83" s="22" t="n"/>
       <c r="J83" s="22" t="n"/>
@@ -11990,9 +11986,9 @@
       <c r="C84" s="22" t="n"/>
       <c r="D84" s="22" t="n"/>
       <c r="E84" s="22" t="n"/>
-      <c r="F84" s="22" t="n"/>
-      <c r="G84" s="22" t="n"/>
-      <c r="H84" s="22" t="n"/>
+      <c r="F84" s="25" t="n"/>
+      <c r="G84" s="25" t="n"/>
+      <c r="H84" s="25" t="n"/>
       <c r="I84" s="22" t="n"/>
       <c r="J84" s="22" t="n"/>
       <c r="K84" s="22" t="n"/>
@@ -12023,9 +12019,9 @@
       <c r="C85" s="22" t="n"/>
       <c r="D85" s="22" t="n"/>
       <c r="E85" s="22" t="n"/>
-      <c r="F85" s="22" t="n"/>
-      <c r="G85" s="22" t="n"/>
-      <c r="H85" s="22" t="n"/>
+      <c r="F85" s="26" t="n"/>
+      <c r="G85" s="26" t="n"/>
+      <c r="H85" s="26" t="n"/>
       <c r="I85" s="22" t="n"/>
       <c r="J85" s="22" t="n"/>
       <c r="K85" s="22" t="n"/>
@@ -12052,18 +12048,18 @@
           <t>14. Comentarios, feedback y seguridad</t>
         </is>
       </c>
-      <c r="B86" s="27" t="n"/>
-      <c r="C86" s="27" t="n"/>
-      <c r="D86" s="27" t="n"/>
-      <c r="E86" s="27" t="n"/>
-      <c r="F86" s="27" t="n"/>
+      <c r="B86" s="22" t="n"/>
+      <c r="C86" s="22" t="n"/>
+      <c r="D86" s="22" t="n"/>
+      <c r="E86" s="22" t="n"/>
+      <c r="F86" s="22" t="n"/>
       <c r="G86" s="22" t="n"/>
       <c r="H86" s="22" t="n"/>
-      <c r="I86" s="22" t="n"/>
-      <c r="J86" s="22" t="n"/>
-      <c r="K86" s="22" t="n"/>
-      <c r="L86" s="22" t="n"/>
-      <c r="M86" s="22" t="n"/>
+      <c r="I86" s="27" t="n"/>
+      <c r="J86" s="27" t="n"/>
+      <c r="K86" s="27" t="n"/>
+      <c r="L86" s="27" t="n"/>
+      <c r="M86" s="27" t="n"/>
       <c r="N86" s="22" t="n"/>
       <c r="O86" s="22" t="n"/>
       <c r="P86" s="22" t="n"/>
@@ -12085,14 +12081,14 @@
           <t>14.1 Comentarios de actividad</t>
         </is>
       </c>
-      <c r="B87" s="28" t="n"/>
+      <c r="B87" s="22" t="n"/>
       <c r="C87" s="22" t="n"/>
       <c r="D87" s="22" t="n"/>
       <c r="E87" s="22" t="n"/>
       <c r="F87" s="22" t="n"/>
       <c r="G87" s="22" t="n"/>
       <c r="H87" s="22" t="n"/>
-      <c r="I87" s="22" t="n"/>
+      <c r="I87" s="28" t="n"/>
       <c r="J87" s="22" t="n"/>
       <c r="K87" s="22" t="n"/>
       <c r="L87" s="22" t="n"/>
@@ -12121,14 +12117,14 @@
       <c r="B88" s="22" t="n"/>
       <c r="C88" s="22" t="n"/>
       <c r="D88" s="22" t="n"/>
-      <c r="E88" s="21" t="n"/>
+      <c r="E88" s="22" t="n"/>
       <c r="F88" s="22" t="n"/>
       <c r="G88" s="22" t="n"/>
       <c r="H88" s="22" t="n"/>
       <c r="I88" s="22" t="n"/>
       <c r="J88" s="22" t="n"/>
       <c r="K88" s="22" t="n"/>
-      <c r="L88" s="22" t="n"/>
+      <c r="L88" s="21" t="n"/>
       <c r="M88" s="22" t="n"/>
       <c r="N88" s="22" t="n"/>
       <c r="O88" s="22" t="n"/>
@@ -12154,14 +12150,14 @@
       <c r="B89" s="22" t="n"/>
       <c r="C89" s="22" t="n"/>
       <c r="D89" s="22" t="n"/>
-      <c r="E89" s="25" t="n"/>
+      <c r="E89" s="22" t="n"/>
       <c r="F89" s="22" t="n"/>
       <c r="G89" s="22" t="n"/>
       <c r="H89" s="22" t="n"/>
       <c r="I89" s="22" t="n"/>
       <c r="J89" s="22" t="n"/>
       <c r="K89" s="22" t="n"/>
-      <c r="L89" s="22" t="n"/>
+      <c r="L89" s="25" t="n"/>
       <c r="M89" s="22" t="n"/>
       <c r="N89" s="22" t="n"/>
       <c r="O89" s="22" t="n"/>
@@ -12184,18 +12180,18 @@
           <t>14.4 Testeo</t>
         </is>
       </c>
-      <c r="B90" s="26" t="n"/>
-      <c r="C90" s="26" t="n"/>
-      <c r="D90" s="26" t="n"/>
-      <c r="E90" s="26" t="n"/>
-      <c r="F90" s="26" t="n"/>
+      <c r="B90" s="22" t="n"/>
+      <c r="C90" s="22" t="n"/>
+      <c r="D90" s="22" t="n"/>
+      <c r="E90" s="22" t="n"/>
+      <c r="F90" s="22" t="n"/>
       <c r="G90" s="22" t="n"/>
       <c r="H90" s="22" t="n"/>
-      <c r="I90" s="22" t="n"/>
-      <c r="J90" s="22" t="n"/>
-      <c r="K90" s="22" t="n"/>
-      <c r="L90" s="22" t="n"/>
-      <c r="M90" s="22" t="n"/>
+      <c r="I90" s="26" t="n"/>
+      <c r="J90" s="26" t="n"/>
+      <c r="K90" s="26" t="n"/>
+      <c r="L90" s="26" t="n"/>
+      <c r="M90" s="26" t="n"/>
       <c r="N90" s="22" t="n"/>
       <c r="O90" s="22" t="n"/>
       <c r="P90" s="22" t="n"/>
@@ -12217,18 +12213,18 @@
           <t>14.5 Documentación</t>
         </is>
       </c>
-      <c r="B91" s="27" t="n"/>
-      <c r="C91" s="27" t="n"/>
-      <c r="D91" s="27" t="n"/>
-      <c r="E91" s="27" t="n"/>
-      <c r="F91" s="27" t="n"/>
+      <c r="B91" s="22" t="n"/>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
+      <c r="E91" s="22" t="n"/>
+      <c r="F91" s="22" t="n"/>
       <c r="G91" s="22" t="n"/>
       <c r="H91" s="22" t="n"/>
-      <c r="I91" s="22" t="n"/>
-      <c r="J91" s="22" t="n"/>
-      <c r="K91" s="22" t="n"/>
-      <c r="L91" s="22" t="n"/>
-      <c r="M91" s="22" t="n"/>
+      <c r="I91" s="27" t="n"/>
+      <c r="J91" s="27" t="n"/>
+      <c r="K91" s="27" t="n"/>
+      <c r="L91" s="27" t="n"/>
+      <c r="M91" s="27" t="n"/>
       <c r="N91" s="22" t="n"/>
       <c r="O91" s="22" t="n"/>
       <c r="P91" s="22" t="n"/>
@@ -12304,9 +12300,9 @@
       <c r="T93" s="22" t="n"/>
       <c r="U93" s="22" t="n"/>
       <c r="V93" s="22" t="n"/>
-      <c r="W93" s="29" t="inlineStr">
-        <is>
-          <t>en curso</t>
+      <c r="W93" s="23" t="inlineStr">
+        <is>
+          <t>completado</t>
         </is>
       </c>
     </row>
@@ -12337,9 +12333,9 @@
       <c r="T94" s="22" t="n"/>
       <c r="U94" s="22" t="n"/>
       <c r="V94" s="22" t="n"/>
-      <c r="W94" s="30" t="inlineStr">
-        <is>
-          <t>sin iniciar</t>
+      <c r="W94" s="29" t="inlineStr">
+        <is>
+          <t>en curso</t>
         </is>
       </c>
     </row>
@@ -12549,8 +12545,8 @@
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="P5:V5"/>
     <mergeCell ref="B4:H4"/>
+    <mergeCell ref="W4:W7"/>
     <mergeCell ref="P4:V4"/>
-    <mergeCell ref="W4:W7"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="B5:H5"/>

</xml_diff>